<commit_message>
source boms by vendor
Claude-Session: https://claude.ai/code/session_01RCYT2QSY7BVZDeTyE9KrC4
</commit_message>
<xml_diff>
--- a/bom/bom-production.xlsx
+++ b/bom/bom-production.xlsx
@@ -446,17 +446,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H29"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="52" customWidth="1" min="1" max="1"/>
+    <col width="56" customWidth="1" min="1" max="1"/>
     <col width="5" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="42" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="52" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="8" max="8"/>
+    <col width="53" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -469,7 +470,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Rev 0.3, 11 x 42 mm 4-layer, sourced from LCSC/JLCPCB. Quantities are per board.</t>
+          <t>Rev 0.3, 11 x 42 mm 4-layer. All parts sourced through JLCPCB assembly (LCSC part numbers). Quantities are per board.</t>
         </is>
       </c>
     </row>
@@ -507,10 +508,15 @@
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>LCSC</t>
+          <t>JLCPCB / LCSC part</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -542,7 +548,12 @@
           <t>C23733</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr"/>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -570,7 +581,12 @@
           <t>C52923</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr"/>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -598,7 +614,12 @@
           <t>C23692971</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr"/>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -626,7 +647,12 @@
           <t>C1525</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr"/>
+      <c r="H8" s="4" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="I8" s="4" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -654,7 +680,12 @@
           <t>C130723</t>
         </is>
       </c>
-      <c r="H9" s="4" t="inlineStr"/>
+      <c r="H9" s="4" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="I9" s="4" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -682,7 +713,12 @@
           <t>C2988369</t>
         </is>
       </c>
-      <c r="H10" s="4" t="inlineStr"/>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -706,7 +742,8 @@
       <c r="E11" s="4" t="inlineStr"/>
       <c r="F11" s="4" t="inlineStr"/>
       <c r="G11" s="4" t="inlineStr"/>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="H11" s="4" t="inlineStr"/>
+      <c r="I11" s="4" t="inlineStr">
         <is>
           <t>bare solder pads - no part to order</t>
         </is>
@@ -738,7 +775,12 @@
           <t>C25905</t>
         </is>
       </c>
-      <c r="H12" s="4" t="inlineStr"/>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
@@ -766,7 +808,12 @@
           <t>C25765</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr"/>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
@@ -794,7 +841,12 @@
           <t>C11702</t>
         </is>
       </c>
-      <c r="H14" s="4" t="inlineStr"/>
+      <c r="H14" s="4" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="I14" s="4" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
@@ -822,7 +874,12 @@
           <t>C25900</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr"/>
+      <c r="H15" s="4" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="I15" s="4" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
@@ -850,7 +907,12 @@
           <t>C26083</t>
         </is>
       </c>
-      <c r="H16" s="4" t="inlineStr"/>
+      <c r="H16" s="4" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="I16" s="4" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -874,7 +936,8 @@
       <c r="E17" s="4" t="inlineStr"/>
       <c r="F17" s="4" t="inlineStr"/>
       <c r="G17" s="4" t="inlineStr"/>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="H17" s="4" t="inlineStr"/>
+      <c r="I17" s="4" t="inlineStr">
         <is>
           <t>bare pad - no part</t>
         </is>
@@ -902,7 +965,8 @@
       <c r="E18" s="4" t="inlineStr"/>
       <c r="F18" s="4" t="inlineStr"/>
       <c r="G18" s="4" t="inlineStr"/>
-      <c r="H18" s="4" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr"/>
+      <c r="I18" s="4" t="inlineStr">
         <is>
           <t>bare pad - no part</t>
         </is>
@@ -930,7 +994,8 @@
       <c r="E19" s="4" t="inlineStr"/>
       <c r="F19" s="4" t="inlineStr"/>
       <c r="G19" s="4" t="inlineStr"/>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="H19" s="4" t="inlineStr"/>
+      <c r="I19" s="4" t="inlineStr">
         <is>
           <t>bare pad - no part</t>
         </is>
@@ -958,7 +1023,8 @@
       <c r="E20" s="4" t="inlineStr"/>
       <c r="F20" s="4" t="inlineStr"/>
       <c r="G20" s="4" t="inlineStr"/>
-      <c r="H20" s="4" t="inlineStr">
+      <c r="H20" s="4" t="inlineStr"/>
+      <c r="I20" s="4" t="inlineStr">
         <is>
           <t>bare pad - no part</t>
         </is>
@@ -999,6 +1065,11 @@
         </is>
       </c>
       <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t>Mouser/DigiKey (consign)</t>
+        </is>
+      </c>
+      <c r="I21" s="4" t="inlineStr">
         <is>
           <t>0 stock at JLC/LCSC - source from Mouser or DigiKey</t>
         </is>
@@ -1030,7 +1101,12 @@
           <t>C967633</t>
         </is>
       </c>
-      <c r="H22" s="4" t="inlineStr"/>
+      <c r="H22" s="4" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="I22" s="4" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
@@ -1058,7 +1134,12 @@
           <t>C424093</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr"/>
+      <c r="H23" s="4" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="I23" s="4" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
@@ -1086,7 +1167,12 @@
           <t>C493453</t>
         </is>
       </c>
-      <c r="H24" s="4" t="inlineStr"/>
+      <c r="H24" s="4" t="inlineStr">
+        <is>
+          <t>JLCPCB</t>
+        </is>
+      </c>
+      <c r="I24" s="4" t="inlineStr"/>
     </row>
     <row r="25"/>
     <row r="26">
@@ -1099,21 +1185,28 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>U1 ISP1807-LR-RS has 0 stock at LCSC/JLCPCB: order from Mouser or DigiKey and consign it, or hand-place.</t>
+          <t>Order the PCB and assembly at jlcpcb.com; upload gerbers, BOM and CPL from production/output/.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>J2 battery pads and TP1/TP2/TP4/TP5 test pads are bare copper, nothing to order.</t>
+          <t>U1 ISP1807-LR-RS is the one exception: 0 stock at JLCPCB/LCSC. Buy it from Mouser or DigiKey and use JLC parts consignment, or hand-place it.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>All passives are 0402 JLC basic parts.</t>
+          <t>J2 battery pads and TP1/TP2/TP4/TP5 test pads are bare copper, nothing to order.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>All passives are 0402 JLC basic parts, no extended-part fee.</t>
         </is>
       </c>
     </row>

</xml_diff>